<commit_message>
paint-factory: redistribute hardware costs into software/on-site sections (totals unchanged: 410k/680k/980k)
</commit_message>
<xml_diff>
--- a/paint-factory/Смета_Лакокрасочный_завод.xlsx
+++ b/paint-factory/Смета_Лакокрасочный_завод.xlsx
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D16"/>
+  <dimension ref="A2:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -745,177 +745,141 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Аппаратное обеспечение (камеры, Edge PC, освещение, кабели)</t>
+          <t>Архитектура ПО, CV-каскад, бэкенд FastAPI</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>140000</v>
+        <v>270000</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>205000</v>
+        <v>350000</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>345000</v>
+        <v>580000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Архитектура ПО, CV-каскад, бэкенд FastAPI</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>170000</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>245000</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>379000</v>
+          <t>Web-панель СБ (Vite + React), SHA-256, JWT-авторизация</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>NAS-архив, Web-панель СБ (Vite+React), SHA-256, JWT</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Он-сайт внедрение: монтаж, калибровка, ПСИ, ОПЭ</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>230000</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>196000</v>
+          <t>Он-сайт внедрение: поставка, монтаж, калибровка, ПСИ, ОПЭ</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>140000</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>330000</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>ИТОГО ПО ТАРИФУ</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>410000</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>680000</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>980000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Управление проектом (Project Management)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>ИТОГО ПО ТАРИФУ</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n">
-        <v>410000</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>680000</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>980000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Срок реализации по договору</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>3 недели</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>5 недель</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>8 недель</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Привязка видео к маркировке</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Попартийная</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Поштучная</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Поштучная + Web-СБ</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Скорость арбитража возвратов</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Ручной поиск в логах</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Выгрузка по QR в 1 клик</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Мгновенный поиск + SHA-256</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Контакты Neat Studio:  Панфилов Семён  ·  +7 985 219-46-04  ·  @pm_neatstudio  ·  s.panfilov@neat-studio.ru</t>
         </is>
@@ -923,7 +887,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
@@ -938,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F25"/>
+  <dimension ref="A2:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1006,422 +970,264 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Аппаратное обеспечение</t>
+          <t>Архитектура ПО и инженерный стек</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B8" s="17" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Промышленная камера Global Shutter (GigE Vision, 30–60 FPS, сенсор исключает «эффект желе»)</t>
+          <t>R&amp;D, проектирование медиа-конвейеров GStreamer и анализ аппаратной части (камеры, оптика, освещение)</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>20 ч</t>
         </is>
       </c>
       <c r="E8" s="18" t="n">
-        <v>45000</v>
+        <v>2500</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>1.1.2</t>
         </is>
       </c>
       <c r="B9" s="17" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Промышленный объектив высокого разрешения (фиксированное фокусное расстояние, ручная юстировка)</t>
+          <t>Разработка слоя компьютерного зрения (CV Core): захват потока через GigE Vision API на Python</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>40 ч</t>
         </is>
       </c>
       <c r="E9" s="18" t="n">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>12000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>1.1.3</t>
         </is>
       </c>
       <c r="B10" s="17" t="n"/>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Контур направленного импульсного LED-освещения (стабилизация контрастности зоны маркировки)</t>
+          <t>Модуль асинхронного сжатия (H.264/H.265) и нарезки логов через FFmpeg; конфигурация Edge PC</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>30 ч</t>
         </is>
       </c>
       <c r="E10" s="18" t="n">
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>15000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>1.1.4</t>
         </is>
       </c>
       <c r="B11" s="17" t="n"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Управляющий компьютер Edge PC (промышленное исполнение, Intel i5/i7, 16 ГБ RAM, Linux Ubuntu)</t>
+          <t>Интеграция модуля сопряжения: обработка сигналов триггера и датчиков положения конвейера на GPIO</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>16 ч</t>
         </is>
       </c>
       <c r="E11" s="18" t="n">
-        <v>55000</v>
+        <v>2500</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>55000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>3.1.5</t>
+          <t>1.1.5</t>
         </is>
       </c>
       <c r="B12" s="17" t="n"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Материалы трассировки и экранированная коммутация конвейера (кабель STP Cat6, разъёмы RJ-45)</t>
+          <t>Лабораторное тестирование: стенд с камерой, освещением, валидация утечек памяти под аптайм Linux</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>1 лот</t>
+          <t>20 ч</t>
         </is>
       </c>
       <c r="E12" s="18" t="n">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>3.1.6</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Индустриальный виброгасящий регулируемый кронштейн надконвейерного монтажа узлов</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>1 шт.</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F13" s="19" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Архитектура ПО и инженерный стек</t>
-        </is>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Пусконаладка и он-сайт интеграция</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>1.2.1</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Управление проектом: архитектурный контроль дорожной карты интеграции, координация поставок</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>20 ч</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>40000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>3.2.1</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B15" s="17" t="n"/>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>R&amp;D и проектирование низкоуровневых медиа-конвейеров во фреймворке GStreamer</t>
+          <t>Шеф-монтаж узлов ПАК: поставка и позиционирование камер, освещения и кронштейнов над линией</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>12 ч</t>
+          <t>1 выезд</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
-        <v>2500</v>
+        <v>44000</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>30000</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>3.2.2</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B16" s="17" t="n"/>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Разработка слоя компьютерного зрения (CV Core): захват потока через GigE Vision API на Python</t>
+          <t>On-Site калибровка CV-скриптов и экспозиции под максимальную скорость движения конвейера</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>24 ч</t>
+          <t>16 ч</t>
         </is>
       </c>
       <c r="E16" s="18" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>48000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>3.2.3</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="B17" s="17" t="n"/>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Разработка модуля асинхронного сжатия (H.264/H.265) и нарезки логов через FFmpeg</t>
+          <t>Проведение приёмо-сдаточных испытаний (ПСИ) системы в течение полной рабочей смены</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>20 ч</t>
+          <t>8 ч</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>2000</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>3.2.4</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Интеграция модуля сопряжения: обработка сигналов триггера и датчиков положения конвейера на GPIO</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>10 ч</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F18" s="19" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>3.2.5</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Лабораторное тестирование: нагрузочный аудит кода и валидация утечек памяти под аптайм Linux</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>15 ч</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>27000</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>Пусконаладка и он-сайт интеграция</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>3.3.1</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Управление проектом (Project Management): архитектурный контроль дорожной карты интеграции</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>15 ч</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F21" s="19" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>3.3.2</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Шеф-монтаж узлов ПАК: механическое позиционирование камер и световых модулей над линией</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>1 выезд</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="n">
-        <v>24000</v>
-      </c>
-      <c r="F22" s="19" t="n">
-        <v>24000</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>3.3.3</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>On-Site калибровка CV-скриптов и экспозиции под максимальную скорость движения конвейера</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>12 ч</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F23" s="19" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>3.3.4</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Проведение приёмо-сдаточных испытаний (ПСИ) системы в течение полной рабочей смены</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>8 ч</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F24" s="19" t="n">
         <v>16000</v>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>ИТОГО ПО ТАРИФУ</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="n"/>
-      <c r="F25" s="8" t="n">
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="20" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="20" t="n"/>
+      <c r="F18" s="8" t="n">
         <v>410000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="15">
     <mergeCell ref="B4:F4"/>
-    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A7:F7"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1434,7 +1240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F22"/>
+  <dimension ref="A2:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1502,147 +1308,147 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Аппаратное обеспечение (Hardware Layer)</t>
+          <t>Архитектура ПО, серверная логика и CV (Software Core)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>2.1.1</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B8" s="17" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Вычислительный узел Edge PC (промышленное исполнение, Intel i7, 16 ГБ RAM, NVMe SSD, Linux)</t>
+          <t>Проектирование реляционной структуры БД PostgreSQL, индексов и бизнес-логики связывания файлов</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>40 ч</t>
         </is>
       </c>
       <c r="E8" s="18" t="n">
-        <v>115000</v>
+        <v>1500</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>115000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>2.1.2</t>
+          <t>1.1.2</t>
         </is>
       </c>
       <c r="B9" s="17" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Промышленная MV-камера высокого разрешения (Global Shutter, 60 FPS, GigE Vision, GPIO-триггер)</t>
+          <t>Разработка асинхронного ядра серверной части на FastAPI; конфигурация Edge PC и сетевого узла</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>90 ч</t>
         </is>
       </c>
       <c r="E9" s="18" t="n">
-        <v>48000</v>
+        <v>1500</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>48000</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>2.1.3</t>
+          <t>1.1.3</t>
         </is>
       </c>
       <c r="B10" s="17" t="n"/>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Контур направленного импульсного LED-освещения высокой интенсивности для стабилизации контраста</t>
+          <t>CV-пайплайн pyzbar / ZXing / OpenCV, подбор и калибровка оптической схемы (камера, объектив, свет)</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>80 ч</t>
         </is>
       </c>
       <c r="E10" s="18" t="n">
-        <v>22000</v>
+        <v>1500</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>22000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>2.1.4</t>
+          <t>1.1.4</t>
         </is>
       </c>
       <c r="B11" s="17" t="n"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Комплект коммутации и экранированной трассировки кабельных трасс конвейера (STP Cat6a, RJ-45)</t>
+          <t>Скрипт автоматической сегментации через FFmpeg и циклической перезаписи архива</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>1 лот</t>
+          <t>28 ч</t>
         </is>
       </c>
       <c r="E11" s="18" t="n">
-        <v>20000</v>
+        <v>1250</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>20000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Архитектура ПО, серверная логика и CV (Software Core)</t>
+          <t>Он-сайт внедрение, калибровка латентности и тесты</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>2.2.1</t>
+          <t>1.2.1</t>
         </is>
       </c>
       <c r="B13" s="17" t="n"/>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Проектирование реляционной структуры БД PostgreSQL, индексов и бизнес-логики связывания файлов</t>
+          <t>Физический шеф-монтаж узлов ПАК: поставка и инсталляция камеры, оптики, освещения, кабельных трасс</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>30 ч</t>
+          <t>48 ч</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
-        <v>1500</v>
+        <v>1667</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>45000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>2.2.2</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B14" s="17" t="n"/>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Разработка асинхронного ядра серверной части на FastAPI (обработка прерываний, API-эндпоинты)</t>
+          <t>Сквозное нагрузочное тестирование пайплайна и оптимизация временных задержек (Latency ≤ 80 мс)</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -1651,197 +1457,89 @@
         </is>
       </c>
       <c r="E14" s="18" t="n">
-        <v>1500</v>
+        <v>1667</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>90000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>2.2.3</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B15" s="17" t="n"/>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Оптимизация CV-пайплайна распознавания QR (параллельная работа pyzbar, ZXing и OpenCV на потоке)</t>
+          <t>Проведение опытно-промышленной эксплуатации (ОПЭ) на конвейере совместно с инженерами завода</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>50 ч</t>
+          <t>64 ч</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
-        <v>1700</v>
+        <v>1250</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>85000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>2.2.4</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="B16" s="17" t="n"/>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Разработка скрипта автоматической сегментации через FFmpeg и циклической перезаписи архива</t>
+          <t>Управление проектом (Project Management): архитектурный контроль, сдача вех по ТЗ, поставки</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>20 ч</t>
+          <t>35 ч</t>
         </is>
       </c>
       <c r="E16" s="18" t="n">
-        <v>1250</v>
+        <v>2000</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Он-сайт внедрение, калибровка латентности и тесты</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>2.3.1</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Физический шеф-монтаж узлов ПАК, калибровка оптических осей камеры и фокусного расстояния</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>24 ч</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="n">
-        <v>1667</v>
-      </c>
-      <c r="F18" s="19" t="n">
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>2.3.2</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Сквозное нагрузочное тестирование пайплайна и оптимизация временных задержек (Latency ≤ 80 мс)</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>36 ч</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="n">
-        <v>1667</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>2.3.3</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Проведение опытно-промышленной эксплуатации (ОПЭ) на конвейере совместно с инженерами завода</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>48 ч</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="n">
-        <v>1250</v>
-      </c>
-      <c r="F20" s="19" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>2.3.4</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Управление проектом (Project Management): архитектурный контроль и сдача вех по ТЗ</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>35 ч</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F21" s="19" t="n">
         <v>70000</v>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>ИТОГО ПО ТАРИФУ</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="8" t="n">
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="20" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="20" t="n"/>
+      <c r="F17" s="8" t="n">
         <v>680000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="14">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1855,7 +1553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F22"/>
+  <dimension ref="A2:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1923,132 +1621,132 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Расширенный аппаратный слой (Hardware Infrastructure)</t>
+          <t>Разработка ПО, криптография и Web-интерфейс (Full Software Stack)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B8" s="17" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Вычислительный узел Edge PC (промышленный ПК, Intel i7, 16 ГБ RAM, NVMe SSD, Linux Ubuntu)</t>
+          <t>Бэкенд FastAPI, модули CV (OpenCV/pyzbar), FFmpeg-нарезка; конфигурация Edge PC и серверного узла</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>120 ч</t>
         </is>
       </c>
       <c r="E8" s="18" t="n">
-        <v>115000</v>
+        <v>1500</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>115000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>1.1.2</t>
         </is>
       </c>
       <c r="B9" s="17" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Выделенный сервер видеоархива NAS (сетевое хранилище, RAID-массив корпоративного класса, 4×4 ТБ)</t>
+          <t>Модуль защиты данных: SHA-256, JWT-авторизация, безопасность логов БД и серверного контура</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>1 компл.</t>
+          <t>60 ч</t>
         </is>
       </c>
       <c r="E9" s="18" t="n">
-        <v>140000</v>
+        <v>1750</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>140000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>1.1.3</t>
         </is>
       </c>
       <c r="B10" s="17" t="n"/>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Промышленная MV-камера (Global Shutter, 60 FPS, GigE Vision, объектив высокого разрешения)</t>
+          <t>Frontend-панель администратора / СБ (Vite + React); подбор и интеграция камер, оптики, освещения</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1 шт.</t>
+          <t>110 ч</t>
         </is>
       </c>
       <c r="E10" s="18" t="n">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>60000</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>1.1.4</t>
         </is>
       </c>
       <c r="B11" s="17" t="n"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Импульсный LED-осветитель и экранированные кабельные трассы STP Cat6 с виброгасящим кронштейном</t>
+          <t>Скрипт репликации и синхронизации с NAS-сервером архивации; конфигурация RAID-массива 4×4 ТБ</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>1 лот</t>
+          <t>50 ч</t>
         </is>
       </c>
       <c r="E11" s="18" t="n">
-        <v>30000</v>
+        <v>1500</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>30000</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Разработка ПО, криптография и Web-интерфейс (Full Software Stack)</t>
+          <t>Он-сайт интеграция, стресс-тесты и ПНР (Enterprise Deployment)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>3.2.1</t>
+          <t>1.2.1</t>
         </is>
       </c>
       <c r="B13" s="17" t="n"/>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Разработка бэкенда на FastAPI, модулей CV (OpenCV/pyzbar) и асинхронной нарезки видеофайлов через FFmpeg</t>
+          <t>Шеф-монтаж: поставка и инсталляция камер, NAS-сервера, оптики, освещения, кабельных трасс; юстировка</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>80 ч</t>
+          <t>72 ч</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
-        <v>1500</v>
+        <v>1667</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>120000</v>
@@ -2057,212 +1755,104 @@
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>3.2.2</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B14" s="17" t="n"/>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Интеграция модуля защиты данных: хэширование файлов SHA-256, авторизация JWT, безопасность логов БД</t>
+          <t>Стресс-тестирование кибербезопасности, нагрузочные испытания RAID и верификация Latency ≤ 80 мс</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>40 ч</t>
+          <t>55 ч</t>
         </is>
       </c>
       <c r="E14" s="18" t="n">
-        <v>1750</v>
+        <v>2000</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>3.2.3</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B15" s="17" t="n"/>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Разработка Frontend-панели администратора / СБ (поиск по ID, плеер, Vite + React, экспорт в 1 клик)</t>
+          <t>Проведение расширенной ОПЭ и ПСИ в течение двух полных смен, обучение операторов завода</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>90 ч</t>
+          <t>60 ч</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>144000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>3.2.4</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="B16" s="17" t="n"/>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Скрипт автоматической репликации данных и синхронизации с NAS-сервером архивации</t>
+          <t>Управление проектом: архитектурный надзор, интеграция с ERP завода, координация поставок</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>30 ч</t>
+          <t>40 ч</t>
         </is>
       </c>
       <c r="E16" s="18" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Он-сайт интеграция, стресс-тесты и ПНР (Enterprise Deployment)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>3.3.1</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Шеф-монтаж, юстировка оптики, калибровка триггеров на GPIO и пусконаладка сетевой топологии</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>40 ч</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="n">
-        <v>1650</v>
-      </c>
-      <c r="F18" s="19" t="n">
-        <v>66000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>3.3.2</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Стресс-тестирование кибербезопасности, нагрузочные испытания RAID и верификация Latency ≤ 80 мс</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>40 ч</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="n">
-        <v>1750</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>3.3.3</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Проведение расширенной ОПЭ и ПСИ в течение двух полных смен, обучение операторов завода</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>40 ч</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F20" s="19" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>3.3.4</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Управление проектом (Project Management): архитектурный надзор, интеграция с ERP завода</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>30 ч</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F21" s="19" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>ИТОГО ПО ТАРИФУ</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="8" t="n">
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="20" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="20" t="n"/>
+      <c r="F17" s="8" t="n">
         <v>980000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="14">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
paint-factory: remove V8 version label from all KP/smeta descriptions
</commit_message>
<xml_diff>
--- a/paint-factory/Смета_Лакокрасочный_завод.xlsx
+++ b/paint-factory/Смета_Лакокрасочный_завод.xlsx
@@ -709,7 +709,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Сводная смета по тарифным планам ПАК V8</t>
+          <t>Сводная смета по тарифным планам ПАК</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Детализированная смета: ПАК V8</t>
+          <t>Детализированная смета: ПАК</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Детализированная смета: ПАК V8</t>
+          <t>Детализированная смета: ПАК</t>
         </is>
       </c>
     </row>
@@ -1568,14 +1568,14 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Детализированная смета: ПАК V8</t>
+          <t>Детализированная смета: ПАК</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Заказчик: Лакокрасочный завод   ·   Тариф: «Корпоративный — Премиум-сборка V8»</t>
+          <t>Заказчик: Лакокрасочный завод   ·   Тариф: «Корпоративный — Премиум-сборка»</t>
         </is>
       </c>
     </row>

</xml_diff>